<commit_message>
test git push/change 2 files test_p1.py & testcase.xlsx:
</commit_message>
<xml_diff>
--- a/case/testcase.xlsx
+++ b/case/testcase.xlsx
@@ -10,7 +10,7 @@
     <sheet name="p2" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1" concurrentCalc="0"/>
 </workbook>
 </file>
 
@@ -819,17 +819,17 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>电性能参数按批次号汇总</t>
+          <t>数据汇总-电性能（RS）</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>/datack/get/halm/summary/charts</t>
+          <t>/datack/common/query/electricalPropertyArgumentQuarter</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>电性能参数按批次号汇总</t>
+          <t>数据汇总-电性能（RS）</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -840,16 +840,13 @@
       <c r="F2" s="4" t="inlineStr">
         <is>
           <t>{
-    "tagsContains": [],
-    "tagsNotContains": [],
-    "lineSideNoList": [
-        "1_1",
-        "1_2"
-    ],
-    "trackNoList": [],
-    "startTime":"${begintime}",
-    "endTime": "${endtime}",
-    "commentList": []
+    "queryParam": {
+        "lineNo": 0,
+        "sideNo": 0,
+        "classId": 0,
+        "startTime": "2024-10-01 00:00:00",
+        "endTime": "2024-12-31 23:59:59"
+    }
 }</t>
         </is>
       </c>

</xml_diff>